<commit_message>
feat: Update existing Sinnoh challenges and xlsx file
- Updated the requirements, unlocks, and gifts for existing extra challenges A 1 through F 3 as specified.
- Reordered challenges alphabetically to keep code maintainable.
- Re-generated the 4_Sinnoh_Data.xlsx file.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/4_Sinnoh_Data.xlsx
+++ b/4_Sinnoh_Data.xlsx
@@ -6982,7 +6982,7 @@
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B287" t="str">
         <v>Iron Island</v>
@@ -7005,7 +7005,7 @@
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B288" t="str">
         <v>Iron Island</v>
@@ -7028,7 +7028,7 @@
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B289" t="str">
         <v>Iron Island</v>
@@ -7051,7 +7051,7 @@
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B290" t="str">
         <v>Iron Island</v>
@@ -7074,7 +7074,7 @@
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B291" t="str">
         <v>Iron Island</v>
@@ -7097,7 +7097,7 @@
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B292" t="str">
         <v>Iron Island</v>
@@ -7120,7 +7120,7 @@
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B293" t="str">
         <v>Iron Island</v>
@@ -9519,7 +9519,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C60"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9826,7 +9826,7 @@
         <v>Earn Mine Badge</v>
       </c>
       <c r="C28" t="str">
-        <v>Unlocks: Route 216, Iron Island</v>
+        <v>Unlocks: Route 216</v>
       </c>
     </row>
     <row r="29">
@@ -9914,7 +9914,7 @@
         <v>{"defeatSinnohChampion":true}</v>
       </c>
       <c r="C36" t="str">
-        <v>Unlocks: Deep Lake Verity, Iron Island, Sendoff Spring, Route 225, Route 224, New Region to Travel, Gift: 2 Masterball</v>
+        <v>Unlocks: Deep Lake Verity, Iron Island, Sendoff Spring, Route 225, Route 224, New Region to Travel, (Extra Challenges B C D E F), Gift: 2 Masterball</v>
       </c>
     </row>
     <row r="37">
@@ -9952,172 +9952,238 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Extra Challenge B 1</v>
+        <v>Extra Challenge A 4</v>
       </c>
       <c r="B40" t="str">
-        <v>Catch 1 Geodude</v>
+        <v>Catch 1 Porygon2</v>
       </c>
       <c r="C40" t="str">
-        <v>Unlocks: Lake Acuity, Gift: 1 Steel Stone</v>
+        <v>Gift: 1 Masterball</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Extra Challenge B 2</v>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B41" t="str">
-        <v>Catch 1 Bibarel</v>
+        <v>Catch 1 Geodude</v>
       </c>
       <c r="C41" t="str">
-        <v>Unlocks: Snowpoint Temple, Gift: 1 Masterball</v>
+        <v>Unlocks: Lake Acuity, Gift: 1 Steel Stone</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Extra Challenge B 3</v>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B42" t="str">
-        <v>Catch 1 Swinub</v>
+        <v>Catch 1 Bibarel</v>
       </c>
       <c r="C42" t="str">
-        <v>Unlocks: Guardian's Cavern, Gift: 1 Ice Stone</v>
+        <v>Unlocks: Snowpoint Temple, Gift: 1 Masterball</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Extra Challenge C 1</v>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B43" t="str">
-        <v>Catch 1 Gastrodon</v>
+        <v>Catch 1 Swinub</v>
       </c>
       <c r="C43" t="str">
-        <v>Unlocks: Deep Lake Valor</v>
+        <v>Unlocks: Guardian's Cavern, Gift: 1 Ice Stone</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Extra Challenge C 2</v>
+        <v>Extra Challenge B 4</v>
       </c>
       <c r="B44" t="str">
-        <v>Catch 1 Lanturn</v>
+        <v>Catch 1 Uxie, Catch 1 Mesprit, Catch 1 Azelf</v>
       </c>
       <c r="C44" t="str">
-        <v>Unlocks: Pastoria Bog, Gift: 1 Masterball</v>
+        <v>Gift: 2 Masterball</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Extra Challenge C 3</v>
+        <v>Extra Challenge C 1</v>
       </c>
       <c r="B45" t="str">
-        <v>Catch 1 Corphish</v>
+        <v>Catch 1 Gastrodon</v>
       </c>
       <c r="C45" t="str">
-        <v>Unlocks: Canalave Sea, Gift: 1 Masterball</v>
+        <v>Unlocks: Deep Lake Valor</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Extra Challenge C 4</v>
+        <v>Extra Challenge C 2</v>
       </c>
       <c r="B46" t="str">
-        <v>Catch 1 Crawdaunt</v>
+        <v>Catch 1 Lanturn</v>
       </c>
       <c r="C46" t="str">
-        <v>Unlocks: Flower Paradise, Gift: 1 Masterball</v>
+        <v>Unlocks: Pastoria Bog, Gift: 1 Masterball</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Extra Challenge D 1</v>
+        <v>Extra Challenge C 3</v>
       </c>
       <c r="B47" t="str">
-        <v>Catch 1 Bibarel</v>
+        <v>Catch 1 Corphish</v>
       </c>
       <c r="C47" t="str">
-        <v>Unlocks: Turnback Cave</v>
+        <v>Unlocks: Canalave Sea, Gift: 1 Masterball</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Extra Challenge D 2</v>
+        <v>Extra Challenge C 4</v>
       </c>
       <c r="B48" t="str">
-        <v>Catch 1 Bronzong</v>
+        <v>Catch 1 Crawdaunt</v>
       </c>
       <c r="C48" t="str">
-        <v>Unlocks: Lunar Isles, Gift: 2 Ghost Stone</v>
+        <v>Unlocks: Flower Paradise, Gift: 1 Masterball</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Extra Challenge E 1</v>
+        <v>Extra Challenge C 5</v>
       </c>
       <c r="B49" t="str">
-        <v>Catch 1 Banette</v>
+        <v>Catch 1 Manaphy, Catch 1 Phione, Catch 1 Shaymin</v>
       </c>
       <c r="C49" t="str">
-        <v>Unlocks: Route 227</v>
+        <v>Gift: 1 Masterball</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Extra Challenge E 2</v>
+        <v>Extra Challenge D 1</v>
       </c>
       <c r="B50" t="str">
-        <v>Catch 1 Banette</v>
+        <v>Catch 1 Bibarel</v>
       </c>
       <c r="C50" t="str">
-        <v>Unlocks: Stark Mountain, Gift: 1 Masterball</v>
+        <v>Unlocks: Turnback Cave</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Extra Challenge E 3</v>
+        <v>Extra Challenge D 2</v>
       </c>
       <c r="B51" t="str">
-        <v>Catch 1 Camerupt</v>
+        <v>Catch 1 Bronzong</v>
       </c>
       <c r="C51" t="str">
-        <v>Unlocks: Continental Depths, Gift: 1 Fire Stone</v>
+        <v>Unlocks: Lunar Isles, Gift: 2 Ghost Stone</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Extra Challenge F 1</v>
+        <v>Extra Challenge D 3</v>
       </c>
       <c r="B52" t="str">
-        <v>Catch 1 Beautifly</v>
+        <v>Catch 1 Cresselia, Catch 1 Darkrai</v>
       </c>
       <c r="C52" t="str">
-        <v>Unlocks: Route 228</v>
+        <v>Gift: 1 Masterball</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Extra Challenge F 2</v>
+        <v>Extra Challenge E 1</v>
       </c>
       <c r="B53" t="str">
-        <v>Catch 1 Cacnea</v>
+        <v>Catch 1 Banette</v>
       </c>
       <c r="C53" t="str">
-        <v>Unlocks: Spear Pillar, Gift: 1 Masterball</v>
+        <v>Unlocks: Route 227</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
+        <v>Extra Challenge E 2</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Catch 1 Banette</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Unlocks: Stark Mountain, Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Extra Challenge E 3</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Catch 1 Camerupt</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Unlocks: Continental Depths, Gift: 1 Fire Stone</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Extra Challenge E 4</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Catch 1 Heatran, Catch 1 Regigigas</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Extra Challenge F 1</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Catch 1 Beautifly</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Unlocks: Route 228</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Extra Challenge F 2</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Catch 1 Cacnea</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Unlocks: Spear Pillar, Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
         <v>Extra Challenge F 3</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B59" t="str">
         <v>Catch 1 Clefairy</v>
       </c>
-      <c r="C54" t="str">
+      <c r="C59" t="str">
         <v>Unlocks: Hall of Origin, Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Extra Challenge F 4</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Catch 1 Arceus, Catch 1 Dialga, Catch 1 Palkia, Catch 1 Giratina</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Gift: 3 Masterball</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C60"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10906,7 +10972,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Challenge 27</v>
+        <v>Challenge 36</v>
       </c>
       <c r="B46" t="str">
         <v>Iron Island</v>

</xml_diff>